<commit_message>
Update employee and student template files: modify Excel templates for improved data import compatibility.
</commit_message>
<xml_diff>
--- a/public/excel/Employee-template.xlsx
+++ b/public/excel/Employee-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tyron\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Academics\Capstone\BPS-LMS-Admin\public\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EDB6E2B1-9140-4D53-8212-1B0A47F6ABD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{75B330D1-BDE5-4CB6-BF9B-78B6911E6A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{92E744CB-172C-4410-AC44-A25B4762E2BC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D1993F5F-8E6D-4076-BE04-F0FC2881C9BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>Data Import Template</t>
   </si>
@@ -44,6 +44,9 @@
     <t>Data:</t>
   </si>
   <si>
+    <t>Employees</t>
+  </si>
+  <si>
     <t>Notes:</t>
   </si>
   <si>
@@ -71,98 +74,83 @@
     <t>Column Labels:</t>
   </si>
   <si>
+    <t>RFID</t>
+  </si>
+  <si>
+    <t>Full_Name</t>
+  </si>
+  <si>
+    <t>Suffix</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
     <t>Column Name:</t>
   </si>
   <si>
+    <t>rfid</t>
+  </si>
+  <si>
+    <t>full_name</t>
+  </si>
+  <si>
+    <t>suffix</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>employee_id</t>
+  </si>
+  <si>
+    <t>employee_role</t>
+  </si>
+  <si>
     <t>Mandatory:</t>
   </si>
   <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
     <t>Type:</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Enum</t>
+  </si>
+  <si>
     <t>Info:</t>
   </si>
   <si>
+    <t xml:space="preserve">Select One of: Male, Female, Prefer not to say </t>
+  </si>
+  <si>
     <t>Start entering data below this line</t>
-  </si>
-  <si>
-    <t>RFID</t>
-  </si>
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Middle Name</t>
-  </si>
-  <si>
-    <t>Last Name</t>
-  </si>
-  <si>
-    <t>suffix</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>rfid</t>
-  </si>
-  <si>
-    <t>first_name</t>
-  </si>
-  <si>
-    <t>middle_name</t>
-  </si>
-  <si>
-    <t>last_name</t>
-  </si>
-  <si>
-    <t>gender</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Enum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select One of: Male, Female, Prefer not to say </t>
-  </si>
-  <si>
-    <t>Employees</t>
-  </si>
-  <si>
-    <t>Suffix</t>
-  </si>
-  <si>
-    <t>Employee ID</t>
-  </si>
-  <si>
-    <t>Position</t>
-  </si>
-  <si>
-    <t>employee_id</t>
-  </si>
-  <si>
-    <t>employee_role</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -174,14 +162,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -207,14 +187,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,210 +523,184 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{088914B6-E621-40AC-902F-6B75EC6AB35B}">
-  <dimension ref="A1:K19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{815050F1-C67C-43AA-855C-DCC0FD00042D}">
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="1" max="1" width="28.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="3" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K14" s="4"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" t="s">
-        <v>26</v>
-      </c>
-      <c r="F15" t="s">
-        <v>20</v>
-      </c>
-      <c r="G15" t="s">
-        <v>27</v>
-      </c>
-      <c r="H15" t="s">
-        <v>28</v>
-      </c>
-      <c r="I15" t="s">
-        <v>38</v>
-      </c>
-      <c r="J15" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" t="s">
-        <v>31</v>
-      </c>
-      <c r="D16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E16" t="s">
-        <v>31</v>
-      </c>
-      <c r="F16" t="s">
-        <v>30</v>
-      </c>
-      <c r="G16" t="s">
-        <v>31</v>
-      </c>
-      <c r="H16" t="s">
-        <v>31</v>
-      </c>
-      <c r="I16" t="s">
-        <v>31</v>
-      </c>
-      <c r="J16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" t="s">
-        <v>29</v>
-      </c>
-      <c r="E17" t="s">
-        <v>29</v>
-      </c>
-      <c r="F17" t="s">
-        <v>29</v>
-      </c>
-      <c r="G17" t="s">
-        <v>32</v>
-      </c>
-      <c r="H17" t="s">
-        <v>29</v>
-      </c>
-      <c r="I17" t="s">
-        <v>29</v>
-      </c>
-      <c r="J17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G18" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>